<commit_message>
Make the Benchmarks tuning check actually able to fire
Health Check row 28 tested Benchmarks!$D$16=0, but that cell always holds a
placeholder threshold, so the row read OK forever. It now reads a real flag
cell, Benchmarks!B28, which ships as PLACEHOLDER and the user changes to TUNED
once the thresholds are the client's own numbers.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Client Reporting Kit/01_Google_Sheets_Reporting_Dashboard.xlsx
+++ b/Client Reporting Kit/01_Google_Sheets_Reporting_Dashboard.xlsx
@@ -31,7 +31,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.00&quot; EGP&quot;"/>
     <numFmt numFmtId="166" formatCode="0.000&quot;x&quot;"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="27">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -177,11 +177,17 @@
     <font>
       <name val="Inter"/>
       <b val="1"/>
+      <color rgb="00B91C1C"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Inter"/>
+      <b val="1"/>
       <color rgb="00111827"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -213,6 +219,11 @@
         <fgColor rgb="00FFF7ED"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -240,7 +251,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -483,6 +494,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -492,7 +506,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
@@ -59180,7 +59194,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -59217,7 +59231,7 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="83" t="inlineStr">
         <is>
-          <t>⚠ The starting numbers below are placeholders so the status columns work on day one — they are not industry truth. Replace them with this client's own trailing 90-day range by month three. A benchmark you didn't measure is a guess, and clients can smell a guess.</t>
+          <t>⚠ The starting numbers below are placeholders so the status columns work on day one — they are not industry truth. Replace them with this client's own trailing 90-day range by month three. A benchmark you didn't measure is a guess, and clients can smell a guess.   •   Once you have replaced them, type TUNED in cell B28 below so Health Check stops flagging this tab.</t>
         </is>
       </c>
     </row>
@@ -59762,6 +59776,23 @@
       <c r="A25" s="89" t="inlineStr">
         <is>
           <t>Lower is better (CPM, CPC, Frequency, Breakeven ROAS): the same ladder, mirrored.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Benchmarks tuning status</t>
+        </is>
+      </c>
+      <c r="B28" s="90" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>Type TUNED here once the thresholds above are this client's own 90-day numbers.</t>
         </is>
       </c>
     </row>
@@ -59851,7 +59882,7 @@
           <t>Zero here means your date cells and your data don't overlap. Start here.</t>
         </is>
       </c>
-      <c r="E6" s="90" t="inlineStr">
+      <c r="E6" s="91" t="inlineStr">
         <is>
           <t>There is no universal good CPM.</t>
         </is>
@@ -59900,7 +59931,7 @@
           <t>First date in the data</t>
         </is>
       </c>
-      <c r="B9" s="91">
+      <c r="B9" s="92">
         <f>IFERROR(MIN(Fundamentals!$A$2:$A$6000),0)</f>
         <v/>
       </c>
@@ -59916,7 +59947,7 @@
           <t>Last date in the data</t>
         </is>
       </c>
-      <c r="B10" s="91">
+      <c r="B10" s="92">
         <f>IFERROR(MAX(Fundamentals!$A$2:$A$6000),0)</f>
         <v/>
       </c>
@@ -59984,7 +60015,7 @@
           <t>Data exists for the selected period</t>
         </is>
       </c>
-      <c r="B17" s="92">
+      <c r="B17" s="93">
         <f>IF('KPI Calc'!$B$10&gt;0,"OK","FIX")</f>
         <v/>
       </c>
@@ -60000,7 +60031,7 @@
           <t>Clicks never exceed impressions</t>
         </is>
       </c>
-      <c r="B18" s="92">
+      <c r="B18" s="93">
         <f>IF('KPI Calc'!$B$12&gt;'KPI Calc'!$B$10,"FIX","OK")</f>
         <v/>
       </c>
@@ -60016,7 +60047,7 @@
           <t>Purchases never exceed clicks</t>
         </is>
       </c>
-      <c r="B19" s="92">
+      <c r="B19" s="93">
         <f>IF('KPI Calc'!$B$16&gt;'KPI Calc'!$B$12,"FIX","OK")</f>
         <v/>
       </c>
@@ -60032,7 +60063,7 @@
           <t>Add to cart never exceeds clicks</t>
         </is>
       </c>
-      <c r="B20" s="92">
+      <c r="B20" s="93">
         <f>IF('KPI Calc'!$B$14&gt;'KPI Calc'!$B$12,"CHECK","OK")</f>
         <v/>
       </c>
@@ -60048,7 +60079,7 @@
           <t>Reach never exceeds impressions</t>
         </is>
       </c>
-      <c r="B21" s="92">
+      <c r="B21" s="93">
         <f>IF('KPI Calc'!$B$11&gt;'KPI Calc'!$B$10,"FIX","OK")</f>
         <v/>
       </c>
@@ -60064,7 +60095,7 @@
           <t>Revenue is present</t>
         </is>
       </c>
-      <c r="B22" s="92">
+      <c r="B22" s="93">
         <f>IF('KPI Calc'!$B$17&lt;=0,"FIX","OK")</f>
         <v/>
       </c>
@@ -60080,7 +60111,7 @@
           <t>Ad spend reconciles to ad-level spend</t>
         </is>
       </c>
-      <c r="B23" s="92">
+      <c r="B23" s="93">
         <f>IF(ABS(SUMIFS('Ad Data'!$G$2:$G$6000,'Ad Data'!$A$2:$A$6000,"&gt;="&amp;'KPI Calc'!$B$4,'Ad Data'!$A$2:$A$6000,"&lt;="&amp;'KPI Calc'!$C$4)-'KPI Calc'!$B$9)/MAX(1,'KPI Calc'!$B$9)&gt;0.05,"CHECK","OK")</f>
         <v/>
       </c>
@@ -60096,7 +60127,7 @@
           <t>Ad-level purchases reconcile</t>
         </is>
       </c>
-      <c r="B24" s="92">
+      <c r="B24" s="93">
         <f>IF(ABS(SUMIFS('Ad Data'!$J$2:$J$6000,'Ad Data'!$A$2:$A$6000,"&gt;="&amp;'KPI Calc'!$B$4,'Ad Data'!$A$2:$A$6000,"&lt;="&amp;'KPI Calc'!$C$4)-'KPI Calc'!$B$16)/MAX(1,'KPI Calc'!$B$16)&gt;0.08,"CHECK","OK")</f>
         <v/>
       </c>
@@ -60112,7 +60143,7 @@
           <t>Business inputs are filled in</t>
         </is>
       </c>
-      <c r="B25" s="92">
+      <c r="B25" s="93">
         <f>IF(OR('KPI Calc'!$J$5&lt;=0,'KPI Calc'!$J$7&lt;=0),"FIX","OK")</f>
         <v/>
       </c>
@@ -60128,7 +60159,7 @@
           <t>Contribution margin is plausible</t>
         </is>
       </c>
-      <c r="B26" s="92">
+      <c r="B26" s="93">
         <f>IF(OR('KPI Calc'!$B$33&lt;=0,'KPI Calc'!$B$33&gt;=1),"CHECK","OK")</f>
         <v/>
       </c>
@@ -60144,7 +60175,7 @@
           <t>No blank platforms in Fundamentals</t>
         </is>
       </c>
-      <c r="B27" s="92">
+      <c r="B27" s="93">
         <f>IF(SUMPRODUCT((Fundamentals!$A$2:$A$6000&lt;&gt;"")*(Fundamentals!$B$2:$B$6000=""))&gt;0,"CHECK","OK")</f>
         <v/>
       </c>
@@ -60160,18 +60191,18 @@
           <t>Benchmarks retuned for this account</t>
         </is>
       </c>
-      <c r="B28" s="92">
-        <f>IF(Benchmarks!$D$16=0,"CHECK","OK")</f>
+      <c r="B28" s="93">
+        <f>IF(Benchmarks!$B$28="TUNED","OK","CHECK")</f>
         <v/>
       </c>
       <c r="C28" s="37" t="inlineStr">
         <is>
-          <t>Until you replace the placeholder thresholds, every Status column is a guess.</t>
+          <t>The Benchmarks tab still holds the shipped placeholders. Replace them with this client's own range, then set Benchmarks!B28 to TUNED.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="28" customHeight="1">
-      <c r="A30" s="93">
+      <c r="A30" s="94">
         <f>IF(COUNTIF(B17:B28,"FIX")&gt;0,"⛔ "&amp;COUNTIF(B17:B28,"FIX")&amp;" check(s) need fixing before you report these numbers.",IF(COUNTIF(B17:B28,"CHECK")&gt;0,"⚠ "&amp;COUNTIF(B17:B28,"CHECK")&amp;" thing(s) to verify. They are usually benign — but verify them.","✅ All "&amp;COUNTA(B17:B28)&amp;" checks passed. This data is safe to report."))</f>
         <v/>
       </c>

</xml_diff>